<commit_message>
Modifiche a tracking checks
</commit_message>
<xml_diff>
--- a/TracingChecks.xlsx
+++ b/TracingChecks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Amedeo\Sviluppo\fuse-angular\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{767F5DA9-A71B-49A9-9AD1-489980DE71AB}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{346DB5E9-A350-400C-B34A-D00F117E0087}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{E91C636A-855F-40D0-AB26-C8EC49A8390A}"/>
+    <workbookView xWindow="696" yWindow="732" windowWidth="15360" windowHeight="8964" xr2:uid="{E91C636A-855F-40D0-AB26-C8EC49A8390A}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -33,10 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>Table name</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Correspondance between fields in old and new version</t>
   </si>
@@ -51,6 +48,18 @@
   </si>
   <si>
     <t>Reports</t>
+  </si>
+  <si>
+    <t>Table name in Old version</t>
+  </si>
+  <si>
+    <t>Json file name in new version</t>
+  </si>
+  <si>
+    <t>Menù</t>
+  </si>
+  <si>
+    <t>Sub-tables</t>
   </si>
 </sst>
 </file>
@@ -101,12 +110,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -421,136 +431,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85886DF3-C6F4-4CF6-A11C-B3E5B02C7355}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="44.5546875" customWidth="1"/>
+    <col min="1" max="1" width="10.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.44140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="44.5546875" style="2" customWidth="1"/>
+    <col min="5" max="9" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Correzioni a tracing checks
</commit_message>
<xml_diff>
--- a/TracingChecks.xlsx
+++ b/TracingChecks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Amedeo\Sviluppo\fuse-angular\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{346DB5E9-A350-400C-B34A-D00F117E0087}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3355BE96-C4C2-4134-AFC2-E352EB145531}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="696" yWindow="732" windowWidth="15360" windowHeight="8964" xr2:uid="{E91C636A-855F-40D0-AB26-C8EC49A8390A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{E91C636A-855F-40D0-AB26-C8EC49A8390A}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Correspondance between fields in old and new version</t>
   </si>
@@ -50,24 +50,41 @@
     <t>Reports</t>
   </si>
   <si>
-    <t>Table name in Old version</t>
-  </si>
-  <si>
     <t>Json file name in new version</t>
   </si>
   <si>
-    <t>Menù</t>
-  </si>
-  <si>
     <t>Sub-tables</t>
+  </si>
+  <si>
+    <t>Attachments</t>
+  </si>
+  <si>
+    <t>Annotations</t>
+  </si>
+  <si>
+    <t>Table name/ menù  in Old version</t>
+  </si>
+  <si>
+    <t>Menù in new version</t>
+  </si>
+  <si>
+    <t>Primary keys of record checked</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -110,13 +127,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -431,45 +449,62 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85886DF3-C6F4-4CF6-A11C-B3E5B02C7355}">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="10.44140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="44.5546875" style="2" customWidth="1"/>
-    <col min="5" max="9" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="19.5546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" style="1" customWidth="1"/>
+    <col min="3" max="4" width="12.109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="34.6640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="7" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.88671875" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="J1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="K1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="I1" s="3" t="s">
+      <c r="L1" s="4" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>